<commit_message>
update comparison table and source xlsx
</commit_message>
<xml_diff>
--- a/ee2.0 vs fenix.xlsx
+++ b/ee2.0 vs fenix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petrsoukup/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petrsoukup/claude/petr-info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F57AA51-EA39-9144-84F3-4D9840D2D6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9D94275-CF02-0E42-9418-6157B290DEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2440" yWindow="920" windowWidth="33720" windowHeight="19220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="920" windowWidth="33720" windowHeight="19220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Porovnání ee2.0 vs Fénix" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="270">
   <si>
     <t>Kapitola</t>
   </si>
@@ -128,9 +128,6 @@
     <t>Produktové štítky</t>
   </si>
   <si>
-    <t>Nastavení stavů (Novinka, Výprodej apod.)</t>
-  </si>
-  <si>
     <t>Možnost uložení a obnovení košíku</t>
   </si>
   <si>
@@ -221,9 +218,6 @@
     <t>24/7 monitoring a notifikace výpadků</t>
   </si>
   <si>
-    <t>GDPR</t>
-  </si>
-  <si>
     <t>Dostupnost podpory</t>
   </si>
   <si>
@@ -363,9 +357,6 @@
   </si>
   <si>
     <t>Výrazně zjednodušen celý proces práce s parametry produktů a variantními parametry.</t>
-  </si>
-  <si>
-    <t>Vlastní barvy štítků v Adminu</t>
   </si>
   <si>
     <t>Košík a objednávkový proces</t>
@@ -816,12 +807,6 @@
     <t>Možnost barevného odlišení stavu objednávky</t>
   </si>
   <si>
-    <t>Stav doručení</t>
-  </si>
-  <si>
-    <t>Nově nastavení barvy stavu</t>
-  </si>
-  <si>
     <t>Číslování objednávky</t>
   </si>
   <si>
@@ -865,6 +850,15 @@
   </si>
   <si>
     <t>2. Střední - Plánujeme dle potřeb klientů</t>
+  </si>
+  <si>
+    <t>Nastavení štítků (Novinka, Výprodej apod.)</t>
+  </si>
+  <si>
+    <t>Tvorba vlastních štítků s možností vlastní barvy v Adminu</t>
+  </si>
+  <si>
+    <t>GDPR, DPA, Přístupnost atd.</t>
   </si>
 </sst>
 </file>
@@ -1082,6 +1076,14 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1091,14 +1093,6 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -1402,7 +1396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39624BD-6325-154A-AB57-B49C9A5453E7}">
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
@@ -1424,56 +1418,56 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="28" t="s">
         <v>82</v>
-      </c>
-      <c r="F1" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
-        <v>84</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F2" s="11"/>
       <c r="G2" s="13"/>
     </row>
     <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="22"/>
+      <c r="A3" s="28"/>
       <c r="B3" s="12" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>87</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>89</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="13"/>
     </row>
     <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="22"/>
+      <c r="A4" s="28"/>
       <c r="B4" s="14" t="s">
         <v>5</v>
       </c>
@@ -1481,16 +1475,16 @@
         <v>6</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F4" s="11"/>
       <c r="G4" s="13"/>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="22"/>
+      <c r="A5" s="28"/>
       <c r="B5" s="14" t="s">
         <v>7</v>
       </c>
@@ -1507,7 +1501,7 @@
       <c r="G5" s="13"/>
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="22"/>
+      <c r="A6" s="28"/>
       <c r="B6" s="14" t="s">
         <v>9</v>
       </c>
@@ -1515,221 +1509,221 @@
         <v>10</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F6" s="11"/>
       <c r="G6" s="13"/>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="22"/>
+      <c r="A7" s="28"/>
       <c r="B7" s="12" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F7" s="11"/>
       <c r="G7" s="13"/>
     </row>
     <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="22"/>
+      <c r="A8" s="28"/>
       <c r="B8" s="14" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F8" s="11"/>
       <c r="G8" s="13"/>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="22"/>
+      <c r="A9" s="28"/>
       <c r="B9" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>205</v>
-      </c>
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="22"/>
+      <c r="A10" s="28"/>
       <c r="B10" s="14" t="s">
         <v>13</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F10" s="11"/>
       <c r="G10" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E11" s="3" t="s">
+    </row>
+    <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="27"/>
+      <c r="B12" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G11" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="21"/>
-      <c r="B12" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>99</v>
-      </c>
       <c r="D12" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="5"/>
     </row>
     <row r="13" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="21"/>
+      <c r="A13" s="27"/>
       <c r="B13" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="21"/>
+      <c r="A14" s="27"/>
       <c r="B14" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="21"/>
+      <c r="A15" s="27"/>
       <c r="B15" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B16" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>102</v>
-      </c>
       <c r="D16" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F16" s="11"/>
       <c r="G16" s="13"/>
     </row>
     <row r="17" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="22"/>
+      <c r="A17" s="28"/>
       <c r="B17" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F17" s="11"/>
       <c r="G17" s="13"/>
     </row>
     <row r="18" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="22"/>
+      <c r="A18" s="28"/>
       <c r="B18" s="14" t="s">
         <v>16</v>
       </c>
@@ -1737,314 +1731,318 @@
         <v>17</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F18" s="11"/>
       <c r="G18" s="13"/>
     </row>
     <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="22"/>
+      <c r="A19" s="28"/>
       <c r="B19" s="14" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="13" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="22"/>
+        <v>198</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A20" s="28"/>
       <c r="B20" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="C20" s="13"/>
+        <v>18</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>19</v>
+      </c>
       <c r="D20" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F20" s="11"/>
       <c r="G20" s="13" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="32" x14ac:dyDescent="0.2">
-      <c r="A21" s="22"/>
-      <c r="B21" s="14" t="s">
-        <v>18</v>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="28"/>
+      <c r="B21" s="12" t="s">
+        <v>20</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F21" s="11"/>
       <c r="G21" s="13" t="s">
-        <v>260</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22" s="22"/>
-      <c r="B22" s="12" t="s">
-        <v>20</v>
+      <c r="A22" s="28"/>
+      <c r="B22" s="14" t="s">
+        <v>22</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F22" s="11"/>
+        <v>94</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>201</v>
+      </c>
       <c r="G22" s="13" t="s">
-        <v>206</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="22"/>
+      <c r="A23" s="28"/>
       <c r="B23" s="14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F23" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="G23" s="13"/>
+    </row>
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="28"/>
+      <c r="B24" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="G24" s="13"/>
+    </row>
+    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="28"/>
+      <c r="B25" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F25" s="11"/>
+      <c r="G25" s="13"/>
+    </row>
+    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="28"/>
+      <c r="B26" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="13" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="22"/>
-      <c r="B24" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G24" s="13"/>
-    </row>
-    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="22"/>
-      <c r="B25" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G25" s="13"/>
-    </row>
-    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="22"/>
-      <c r="B26" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>208</v>
-      </c>
       <c r="D26" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F26" s="11"/>
-      <c r="G26" s="13"/>
+      <c r="G26" s="13" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="27" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="22"/>
+      <c r="A27" s="28"/>
       <c r="B27" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>107</v>
-      </c>
+        <v>254</v>
+      </c>
+      <c r="C27" s="13"/>
       <c r="D27" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F27" s="11"/>
       <c r="G27" s="13" t="s">
-        <v>108</v>
+        <v>256</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="22"/>
+      <c r="A28" s="28"/>
       <c r="B28" s="14" t="s">
-        <v>259</v>
-      </c>
-      <c r="C28" s="13"/>
+        <v>29</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>267</v>
+      </c>
       <c r="D28" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F28" s="11"/>
       <c r="G28" s="13" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="22"/>
-      <c r="B29" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C29" s="13" t="s">
+      <c r="A29" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E29" s="22" t="s">
+        <v>208</v>
+      </c>
+      <c r="F29" s="3"/>
+      <c r="G29" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="27"/>
+      <c r="B30" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D30" s="3">
+        <v>4</v>
+      </c>
+      <c r="E30" s="22">
+        <v>3</v>
+      </c>
+      <c r="F30" s="3"/>
+      <c r="G30" s="5"/>
+    </row>
+    <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A31" s="27"/>
+      <c r="B31" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="G31" s="5"/>
+    </row>
+    <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32" s="27"/>
+      <c r="B32" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D29" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F29" s="11"/>
-      <c r="G29" s="13" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C30" s="5"/>
-      <c r="D30" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E30" s="25" t="s">
-        <v>211</v>
-      </c>
-      <c r="F30" s="3"/>
-      <c r="G30" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31" s="21"/>
-      <c r="B31" s="6" t="s">
+      <c r="D32" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F32" s="3"/>
+      <c r="G32" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="D31" s="3">
-        <v>4</v>
-      </c>
-      <c r="E31" s="25">
-        <v>3</v>
-      </c>
-      <c r="F31" s="3"/>
-      <c r="G31" s="5"/>
-    </row>
-    <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="21"/>
-      <c r="B32" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="G32" s="5"/>
     </row>
     <row r="33" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="21"/>
+      <c r="A33" s="27"/>
       <c r="B33" s="6" t="s">
-        <v>115</v>
+        <v>31</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>86</v>
+        <v>208</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A34" s="27"/>
+      <c r="B34" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="21"/>
-      <c r="B34" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="D34" s="3" t="s">
-        <v>91</v>
+        <v>208</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="F34" s="3"/>
+        <v>94</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>201</v>
+      </c>
       <c r="G34" s="5" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A35" s="21"/>
+      <c r="A35" s="27"/>
       <c r="B35" s="6" t="s">
         <v>118</v>
       </c>
@@ -2052,115 +2050,113 @@
         <v>119</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>211</v>
+        <v>84</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A36" s="21"/>
+      <c r="A36" s="27"/>
       <c r="B36" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>122</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="C36" s="5"/>
       <c r="D36" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>192</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="F36" s="3"/>
       <c r="G36" s="5" t="s">
-        <v>123</v>
+        <v>251</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="21"/>
+      <c r="A37" s="27"/>
       <c r="B37" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A38" s="21"/>
+      <c r="A38" s="27"/>
       <c r="B38" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="C38" s="5"/>
+      <c r="C38" s="5" t="s">
+        <v>258</v>
+      </c>
       <c r="D38" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F38" s="3"/>
-      <c r="G38" s="5" t="s">
-        <v>258</v>
-      </c>
+      <c r="G38" s="5"/>
     </row>
     <row r="39" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A39" s="21"/>
+      <c r="A39" s="27"/>
       <c r="B39" s="6" t="s">
-        <v>262</v>
+        <v>33</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>263</v>
+        <v>34</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F39" s="3"/>
-      <c r="G39" s="5"/>
+        <v>94</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="40" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A40" s="21"/>
-      <c r="B40" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="G40" s="5" t="s">
+      <c r="A40" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>124</v>
       </c>
+      <c r="D40" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F40" s="11"/>
+      <c r="G40" s="13" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="41" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A41" s="23" t="s">
-        <v>125</v>
-      </c>
+      <c r="A41" s="29"/>
       <c r="B41" s="14" t="s">
         <v>126</v>
       </c>
@@ -2168,379 +2164,381 @@
         <v>127</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F41" s="11"/>
       <c r="G41" s="13" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42" s="29"/>
+      <c r="B42" s="14" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A42" s="23"/>
-      <c r="B42" s="14" t="s">
+      <c r="C42" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="C42" s="13" t="s">
-        <v>130</v>
-      </c>
       <c r="D42" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F42" s="11"/>
       <c r="G42" s="13" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A43" s="29"/>
+      <c r="B43" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="D43" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F43" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="G43" s="13" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A44" s="29"/>
+      <c r="B44" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="D44" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E44" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F44" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="G44" s="13"/>
+    </row>
+    <row r="45" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A45" s="29"/>
+      <c r="B45" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="D45" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F45" s="17"/>
+      <c r="G45" s="13" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" s="23"/>
-      <c r="B43" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="D43" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F43" s="11"/>
-      <c r="G43" s="13" t="s">
+    <row r="46" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A46" s="29"/>
+      <c r="B46" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="C46" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="D46" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="E46" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="F46" s="11"/>
+      <c r="G46" s="20" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A47" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="B47" s="14" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="23"/>
-      <c r="B44" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="D44" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E44" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F44" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="G44" s="13" t="s">
+      <c r="C47" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="D47" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E47" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F47" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="G47" s="13"/>
+    </row>
+    <row r="48" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A48" s="28"/>
+      <c r="B48" s="14" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A45" s="23"/>
-      <c r="B45" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="C45" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E45" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F45" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="G45" s="13"/>
-    </row>
-    <row r="46" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A46" s="23"/>
-      <c r="B46" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="C46" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="D46" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="E46" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="F46" s="17"/>
-      <c r="G46" s="13" t="s">
+      <c r="C48" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="D48" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E48" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F48" s="11"/>
+      <c r="G48" s="13"/>
+    </row>
+    <row r="49" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A49" s="28"/>
+      <c r="B49" s="14" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A47" s="23"/>
-      <c r="B47" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="C47" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="D47" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="E47" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="F47" s="11"/>
-      <c r="G47" s="20" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A48" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="B48" s="14" t="s">
-        <v>216</v>
-      </c>
-      <c r="C48" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="D48" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E48" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F48" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="G48" s="13"/>
-    </row>
-    <row r="49" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A49" s="22"/>
-      <c r="B49" s="14" t="s">
-        <v>217</v>
-      </c>
       <c r="C49" s="13" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F49" s="11"/>
       <c r="G49" s="13"/>
     </row>
     <row r="50" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A50" s="22"/>
+      <c r="A50" s="28"/>
       <c r="B50" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="C50" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="C50" s="13" t="s">
+      <c r="D50" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F50" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="G50" s="13"/>
+    </row>
+    <row r="51" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A51" s="28"/>
+      <c r="B51" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E51" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="G51" s="13"/>
+    </row>
+    <row r="52" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A52" s="28"/>
+      <c r="B52" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D52" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E52" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F52" s="11"/>
+      <c r="G52" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="D50" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E50" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="F50" s="11"/>
-      <c r="G50" s="13"/>
-    </row>
-    <row r="51" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A51" s="22"/>
-      <c r="B51" s="14" t="s">
-        <v>220</v>
-      </c>
-      <c r="C51" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="D51" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="E51" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F51" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G51" s="13"/>
-    </row>
-    <row r="52" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A52" s="22"/>
-      <c r="B52" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="C52" s="13" t="s">
+    </row>
+    <row r="53" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A53" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="D52" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="E52" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F52" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G52" s="13"/>
-    </row>
-    <row r="53" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A53" s="22"/>
-      <c r="B53" s="14" t="s">
-        <v>223</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D53" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E53" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F53" s="11"/>
-      <c r="G53" s="13" t="s">
-        <v>224</v>
-      </c>
+      <c r="C53" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F53" s="3"/>
+      <c r="G53" s="5"/>
     </row>
     <row r="54" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A54" s="21" t="s">
-        <v>143</v>
-      </c>
+      <c r="A54" s="27"/>
       <c r="B54" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="5"/>
     </row>
     <row r="55" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A55" s="21"/>
+      <c r="A55" s="27"/>
       <c r="B55" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G55" s="5"/>
+    </row>
+    <row r="56" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A56" s="27"/>
+      <c r="B56" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C56" s="5"/>
+      <c r="D56" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="G56" s="5"/>
+    </row>
+    <row r="57" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A57" s="27"/>
+      <c r="B57" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="G57" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F55" s="3"/>
-      <c r="G55" s="5"/>
-    </row>
-    <row r="56" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A56" s="21"/>
-      <c r="B56" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G56" s="5"/>
-    </row>
-    <row r="57" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A57" s="21"/>
-      <c r="B57" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="C57" s="5"/>
-      <c r="D57" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="G57" s="5"/>
     </row>
     <row r="58" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A58" s="21"/>
+      <c r="A58" s="27"/>
       <c r="B58" s="6" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="G58" s="5" t="s">
-        <v>234</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="G58" s="5"/>
     </row>
     <row r="59" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A59" s="21"/>
+      <c r="A59" s="27"/>
       <c r="B59" s="6" t="s">
-        <v>227</v>
+        <v>36</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>228</v>
+        <v>141</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="G59" s="5"/>
     </row>
     <row r="60" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A60" s="21"/>
-      <c r="B60" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C60" s="5" t="s">
+      <c r="A60" s="28" t="s">
+        <v>142</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C60" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="D60" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G60" s="5"/>
+      <c r="D60" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E60" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F60" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="G60" s="13" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="61" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A61" s="22" t="s">
-        <v>145</v>
-      </c>
+      <c r="A61" s="28"/>
       <c r="B61" s="14" t="s">
         <v>146</v>
       </c>
@@ -2548,20 +2546,18 @@
         <v>147</v>
       </c>
       <c r="D61" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F61" s="11" t="s">
-        <v>192</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="F61" s="11"/>
       <c r="G61" s="13" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A62" s="22"/>
+      <c r="A62" s="28"/>
       <c r="B62" s="14" t="s">
         <v>149</v>
       </c>
@@ -2569,37 +2565,37 @@
         <v>150</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F62" s="11"/>
       <c r="G62" s="13" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A63" s="28"/>
+      <c r="B63" s="14" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A63" s="22"/>
-      <c r="B63" s="14" t="s">
+      <c r="C63" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="C63" s="13" t="s">
-        <v>153</v>
-      </c>
       <c r="D63" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F63" s="11"/>
       <c r="G63" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A64" s="22"/>
+      <c r="A64" s="28"/>
       <c r="B64" s="14" t="s">
         <v>154</v>
       </c>
@@ -2607,267 +2603,267 @@
         <v>155</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F64" s="11"/>
-      <c r="G64" s="13" t="s">
+      <c r="G64" s="13"/>
+    </row>
+    <row r="65" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="28"/>
+      <c r="B65" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="C65" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="D65" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E65" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F65" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="G65" s="13"/>
+    </row>
+    <row r="66" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A66" s="28"/>
+      <c r="B66" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="C66" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="D66" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E66" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F66" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="G66" s="13" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="28"/>
+      <c r="B67" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C67" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D67" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E67" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F67" s="11"/>
+      <c r="G67" s="13" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="27" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A65" s="22"/>
-      <c r="B65" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="C65" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="D65" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E65" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F65" s="11"/>
-      <c r="G65" s="13"/>
-    </row>
-    <row r="66" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A66" s="22"/>
-      <c r="B66" s="14" t="s">
-        <v>242</v>
-      </c>
-      <c r="C66" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="D66" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="E66" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F66" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="G66" s="13"/>
-    </row>
-    <row r="67" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A67" s="22"/>
-      <c r="B67" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="C67" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="D67" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E67" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F67" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="G67" s="13" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A68" s="22"/>
-      <c r="B68" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C68" s="13" t="s">
+      <c r="B68" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D68" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="E68" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F68" s="11"/>
-      <c r="G68" s="13" t="s">
+      <c r="C68" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F68" s="3"/>
+      <c r="G68" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A69" s="27"/>
+      <c r="B69" s="6" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A69" s="21" t="s">
-        <v>159</v>
-      </c>
-      <c r="B69" s="6" t="s">
+      <c r="C69" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G69" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A70" s="27"/>
+      <c r="B70" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C69" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F69" s="3"/>
-      <c r="G69" s="5" t="s">
+      <c r="C70" s="5" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A70" s="21"/>
-      <c r="B70" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="C70" s="5" t="s">
-        <v>241</v>
-      </c>
       <c r="D70" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F70" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G70" s="5" t="s">
-        <v>239</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="F70" s="3"/>
+      <c r="G70" s="5"/>
     </row>
     <row r="71" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A71" s="21"/>
+      <c r="A71" s="27"/>
       <c r="B71" s="6" t="s">
         <v>44</v>
       </c>
       <c r="C71" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F71" s="3"/>
+      <c r="G71" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A72" s="27"/>
+      <c r="B72" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G72" s="5"/>
+    </row>
+    <row r="73" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A73" s="27"/>
+      <c r="B73" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="G73" s="5"/>
+    </row>
+    <row r="74" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A74" s="27"/>
+      <c r="B74" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A75" s="27"/>
+      <c r="B75" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C75" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="D71" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F71" s="3"/>
-      <c r="G71" s="5"/>
-    </row>
-    <row r="72" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A72" s="21"/>
-      <c r="B72" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F72" s="3"/>
-      <c r="G72" s="5" t="s">
+      <c r="D75" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F75" s="3"/>
+      <c r="G75" s="5"/>
+    </row>
+    <row r="76" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A76" s="27"/>
+      <c r="B76" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C76" s="5" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A73" s="21"/>
-      <c r="B73" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C73" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D73" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E73" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F73" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G73" s="5"/>
-    </row>
-    <row r="74" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A74" s="21"/>
-      <c r="B74" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C74" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E74" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F74" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="G74" s="5"/>
-    </row>
-    <row r="75" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A75" s="21"/>
-      <c r="B75" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C75" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D75" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E75" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F75" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G75" s="5" t="s">
+      <c r="D76" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F76" s="3"/>
+      <c r="G76" s="5" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A77" s="27"/>
+      <c r="B77" s="6" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A76" s="21"/>
-      <c r="B76" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C76" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E76" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F76" s="3"/>
-      <c r="G76" s="5"/>
-    </row>
-    <row r="77" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A77" s="21"/>
-      <c r="B77" s="6" t="s">
+      <c r="C77" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="C77" s="5" t="s">
-        <v>163</v>
-      </c>
       <c r="D77" s="3" t="s">
-        <v>142</v>
+        <v>84</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>141</v>
+        <v>84</v>
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="5" t="s">
-        <v>244</v>
+        <v>163</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A78" s="21"/>
+      <c r="A78" s="27"/>
       <c r="B78" s="6" t="s">
         <v>164</v>
       </c>
@@ -2875,206 +2871,206 @@
         <v>165</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="5" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A79" s="27"/>
+      <c r="B79" s="6" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A79" s="21"/>
-      <c r="B79" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C79" s="5" t="s">
-        <v>168</v>
-      </c>
+      <c r="C79" s="5"/>
       <c r="D79" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A80" s="21"/>
+      <c r="A80" s="27"/>
       <c r="B80" s="6" t="s">
-        <v>169</v>
+        <v>249</v>
       </c>
       <c r="C80" s="5"/>
       <c r="D80" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F80" s="3"/>
-      <c r="G80" s="5" t="s">
-        <v>246</v>
-      </c>
+      <c r="G80" s="5"/>
     </row>
     <row r="81" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A81" s="21"/>
+      <c r="A81" s="27"/>
       <c r="B81" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="C81" s="5"/>
+        <v>50</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="D81" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F81" s="3"/>
-      <c r="G81" s="5"/>
+      <c r="G81" s="5" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="82" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A82" s="21"/>
-      <c r="B82" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C82" s="5" t="s">
+      <c r="A82" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B82" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D82" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E82" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F82" s="3"/>
-      <c r="G82" s="5" t="s">
+      <c r="C82" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D82" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E82" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F82" s="11"/>
+      <c r="G82" s="13"/>
+    </row>
+    <row r="83" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A83" s="28"/>
+      <c r="B83" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C83" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D83" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E83" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F83" s="11"/>
+      <c r="G83" s="13" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A84" s="28"/>
+      <c r="B84" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C84" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="D84" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E84" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F84" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="G84" s="13" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="83" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A83" s="22" t="s">
-        <v>171</v>
-      </c>
-      <c r="B83" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C83" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="D83" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E83" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F83" s="11"/>
-      <c r="G83" s="13"/>
-    </row>
-    <row r="84" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A84" s="22"/>
-      <c r="B84" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C84" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="D84" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E84" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F84" s="11"/>
-      <c r="G84" s="13" t="s">
-        <v>172</v>
-      </c>
-    </row>
     <row r="85" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A85" s="22"/>
+      <c r="A85" s="28"/>
       <c r="B85" s="14" t="s">
         <v>57</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>247</v>
+        <v>171</v>
       </c>
       <c r="D85" s="11" t="s">
-        <v>86</v>
+        <v>172</v>
       </c>
       <c r="E85" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F85" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G85" s="13" t="s">
-        <v>173</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="F85" s="11"/>
+      <c r="G85" s="13"/>
     </row>
     <row r="86" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A86" s="22"/>
+      <c r="A86" s="28"/>
       <c r="B86" s="14" t="s">
         <v>58</v>
       </c>
       <c r="C86" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D86" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E86" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F86" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="G86" s="13" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A87" s="28"/>
+      <c r="B87" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="C87" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="D87" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E87" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F87" s="11"/>
+      <c r="G87" s="13" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A88" s="27" t="s">
+        <v>173</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F88" s="3"/>
+      <c r="G88" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="D86" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="E86" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="F86" s="11"/>
-      <c r="G86" s="13"/>
-    </row>
-    <row r="87" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A87" s="22"/>
-      <c r="B87" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="C87" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="D87" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E87" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F87" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="G87" s="13" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A88" s="22"/>
-      <c r="B88" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C88" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="D88" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E88" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F88" s="11"/>
-      <c r="G88" s="13" t="s">
-        <v>249</v>
-      </c>
     </row>
     <row r="89" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A89" s="21" t="s">
-        <v>176</v>
-      </c>
+      <c r="A89" s="27"/>
       <c r="B89" s="6" t="s">
         <v>62</v>
       </c>
@@ -3082,18 +3078,18 @@
         <v>63</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F89" s="3"/>
       <c r="G89" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A90" s="21"/>
+      <c r="A90" s="27"/>
       <c r="B90" s="6" t="s">
         <v>64</v>
       </c>
@@ -3101,39 +3097,39 @@
         <v>65</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="F90" s="3"/>
       <c r="G90" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A91" s="28" t="s">
+        <v>177</v>
+      </c>
+      <c r="B91" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C91" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D91" s="11" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="91" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A91" s="21"/>
-      <c r="B91" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C91" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E91" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F91" s="3"/>
-      <c r="G91" s="5" t="s">
+      <c r="E91" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="F91" s="11"/>
+      <c r="G91" s="13" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A92" s="22" t="s">
-        <v>180</v>
-      </c>
+      <c r="A92" s="28"/>
       <c r="B92" s="14" t="s">
         <v>68</v>
       </c>
@@ -3141,18 +3137,18 @@
         <v>69</v>
       </c>
       <c r="D92" s="11" t="s">
-        <v>181</v>
+        <v>89</v>
       </c>
       <c r="E92" s="11" t="s">
-        <v>181</v>
+        <v>89</v>
       </c>
       <c r="F92" s="11"/>
       <c r="G92" s="13" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A93" s="22"/>
+      <c r="A93" s="28"/>
       <c r="B93" s="14" t="s">
         <v>70</v>
       </c>
@@ -3160,77 +3156,77 @@
         <v>71</v>
       </c>
       <c r="D93" s="11" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E93" s="11" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="F93" s="11"/>
-      <c r="G93" s="13" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A94" s="22"/>
-      <c r="B94" s="14" t="s">
+      <c r="G93" s="13"/>
+    </row>
+    <row r="94" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A94" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="B94" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C94" s="13" t="s">
+      <c r="C94" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D94" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E94" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="F94" s="11"/>
-      <c r="G94" s="13"/>
-    </row>
-    <row r="95" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="21" t="s">
-        <v>184</v>
-      </c>
+      <c r="D94" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="E94" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F94" s="3"/>
+      <c r="G94" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A95" s="27"/>
       <c r="B95" s="6" t="s">
         <v>74</v>
       </c>
       <c r="C95" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E95" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F95" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="G95" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A96" s="27"/>
+      <c r="B96" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D95" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E95" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F95" s="3"/>
-      <c r="G95" s="5" t="s">
+      <c r="C96" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E96" s="3" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="96" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A96" s="21"/>
-      <c r="B96" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C96" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="D96" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E96" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F96" s="3" t="s">
-        <v>207</v>
-      </c>
+      <c r="F96" s="3"/>
       <c r="G96" s="5" t="s">
-        <v>187</v>
+        <v>260</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A97" s="21"/>
+      <c r="A97" s="27"/>
       <c r="B97" s="6" t="s">
         <v>77</v>
       </c>
@@ -3238,80 +3234,61 @@
         <v>78</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="F97" s="3"/>
+        <v>94</v>
+      </c>
+      <c r="F97" s="3" t="s">
+        <v>201</v>
+      </c>
       <c r="G97" s="5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A99" s="24" t="s">
+        <v>264</v>
+      </c>
+      <c r="B99" s="23" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A98" s="21"/>
-      <c r="B98" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C98" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D98" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E98" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F98" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="G98" s="5" t="s">
-        <v>189</v>
-      </c>
-    </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A100" s="27" t="s">
-        <v>269</v>
-      </c>
-      <c r="B100" s="26" t="s">
-        <v>270</v>
+      <c r="A100" s="25" t="s">
+        <v>261</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A101" s="28" t="s">
+      <c r="A101" s="26"/>
+      <c r="B101" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="B101" s="6" t="s">
-        <v>268</v>
-      </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A102" s="29"/>
+      <c r="A102" s="26"/>
       <c r="B102" s="6" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A103" s="29"/>
-      <c r="B103" s="6" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A95:A98"/>
+    <mergeCell ref="A94:A97"/>
     <mergeCell ref="A2:A10"/>
     <mergeCell ref="A11:A15"/>
-    <mergeCell ref="A16:A29"/>
-    <mergeCell ref="A30:A40"/>
-    <mergeCell ref="A48:A53"/>
-    <mergeCell ref="A54:A60"/>
-    <mergeCell ref="A41:A47"/>
-    <mergeCell ref="A61:A68"/>
-    <mergeCell ref="A69:A82"/>
-    <mergeCell ref="A83:A88"/>
-    <mergeCell ref="A89:A91"/>
-    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="A16:A28"/>
+    <mergeCell ref="A29:A39"/>
+    <mergeCell ref="A47:A52"/>
+    <mergeCell ref="A53:A59"/>
+    <mergeCell ref="A40:A46"/>
+    <mergeCell ref="A60:A67"/>
+    <mergeCell ref="A68:A81"/>
+    <mergeCell ref="A82:A87"/>
+    <mergeCell ref="A88:A90"/>
+    <mergeCell ref="A91:A93"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>